<commit_message>
examples: rigenera output dopo passaggio a LIFO per conto
Esempi rigenerati via 'python scripts/gen_examples.py' dopo il
cambio del metodo di lot matching in forex_gains.

- mascetti/2024: il numero di RT forex lines cambia; la netta forex
  passa a -176.85 EUR per l'anno.
- mascetti/2025: RT forex lines passano da 10 a 2; la netta forex
  passa a -1536.82 EUR.
- magnotta + mosconi: variazioni minime sui PDF/XLSX (solo metadata
  ZIP/build), YAML invariate perche' non superano la soglia valutaria
  e non hanno mai entries forex.
</commit_message>
<xml_diff>
--- a/examples/mascetti/decaf_2024.xlsx
+++ b/examples/mascetti/decaf_2024.xlsx
@@ -574,7 +574,7 @@
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>714.4299999999999</v>
+        <v>749.83</v>
       </c>
     </row>
     <row r="15">
@@ -1725,7 +1725,7 @@
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="35" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
@@ -1973,7 +1973,7 @@
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Plusvalenza valutaria (FIFO USD)</t>
+          <t>Plusvalenza valutaria USD (LIFO per conto)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -2022,12 +2022,12 @@
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Plusvalenza valutaria (FIFO USD)</t>
+          <t>Plusvalenza valutaria USD (LIFO per conto)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2024-02-07</t>
+          <t>2024-09-10</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -2042,10 +2042,10 @@
         <v>1477.7</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>1531.18</v>
+        <v>1495.78</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>-53.48</v>
+        <v>-18.08</v>
       </c>
       <c r="J6" t="n">
         <v>1.1166</v>
@@ -2079,7 +2079,7 @@
         </is>
       </c>
       <c r="I8" s="4" t="n">
-        <v>714.4299999999999</v>
+        <v>749.83</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Release 0.3.4: fix cost basis RSU (Valore Normale vs W-2 USA)
Fix fiscale sostanziale per chi ha RSU su Schwab. Lo Schwab Year-End
Summary riporta come "Cost Basis" il W-2 US basis — il prezzo di
chiusura del giorno di vest, base per il 1099-B americano. Per la
dichiarazione italiana il costo riconosciuto e' invece il Valore
Normale ex art. 9 c. 4 lett. a) TUIR (media aritmetica del mese
precedente al vest) tassato come reddito di lavoro sulla CU: esposto
da Schwab come "ITA FMV" sull'Annual Withholding Statement. Usando
il dato sbagliato le plusvalenze RT risultavano sistematicamente
sottostimate (o artificialmente in minus) per titoli in uptrend nel
mese pre-vest. Decaf ora sostituisce il cost basis con qty × ITA FMV
quando acquisition_date matcha un vest date noto.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/mascetti/decaf_2024.xlsx
+++ b/examples/mascetti/decaf_2024.xlsx
@@ -1958,10 +1958,10 @@
         </is>
       </c>
       <c r="L4" s="4" t="n">
-        <v>175</v>
+        <v>125</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>158.47</v>
+        <v>113.19</v>
       </c>
     </row>
     <row r="5">
@@ -2011,10 +2011,10 @@
         </is>
       </c>
       <c r="L5" s="4" t="n">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="M5" s="4" t="n">
-        <v>22.64</v>
+        <v>13.58</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
Release 0.3.5: controllo coerenza RSU contro CU in tutti gli output
decaf report ora stampa e include in YAML/XLSX/PDF il totale del
reddito RSU tassato nell'anno (ITA FMV x net shares al cambio BCE
vest-day) come sanity-check contro il punto 1 della Certificazione
Unica "Redditi di lavoro dipendente". Complementa il fix cost basis
della 0.3.4: ora l'utente puo' verificare a occhio che decaf stia
usando come costo lo stesso valore tassato da Meta in busta paga.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/mascetti/decaf_2024.xlsx
+++ b/examples/mascetti/decaf_2024.xlsx
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -40,6 +40,10 @@
     <font>
       <b val="1"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="3">
@@ -68,12 +72,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
@@ -443,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:D27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -648,7 +653,47 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" s="2" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Controllo coerenza RSU (art. 9 c. 4 TUIR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Vest events nell'anno</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Reddito RSU tassato (EUR)</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="n">
+        <v>4727.27</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Cross-check: deve essere sottoinsieme del punto 1 CU "Redditi di lavoro dipendente". Differenza = stipendio + bonus.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A27:D27"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -684,97 +729,97 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>Cod.</t>
         </is>
       </c>
-      <c r="B1" s="5" t="inlineStr">
+      <c r="B1" s="6" t="inlineStr">
         <is>
           <t>ISIN</t>
         </is>
       </c>
-      <c r="C1" s="5" t="inlineStr">
+      <c r="C1" s="6" t="inlineStr">
         <is>
           <t>Simbolo</t>
         </is>
       </c>
-      <c r="D1" s="5" t="inlineStr">
+      <c r="D1" s="6" t="inlineStr">
         <is>
           <t>Azienda</t>
         </is>
       </c>
-      <c r="E1" s="5" t="inlineStr">
+      <c r="E1" s="6" t="inlineStr">
         <is>
           <t>Descrizione</t>
         </is>
       </c>
-      <c r="F1" s="5" t="inlineStr">
+      <c r="F1" s="6" t="inlineStr">
         <is>
           <t>Valuta</t>
         </is>
       </c>
-      <c r="G1" s="5" t="inlineStr">
+      <c r="G1" s="6" t="inlineStr">
         <is>
           <t>Paese</t>
         </is>
       </c>
-      <c r="H1" s="5" t="inlineStr">
+      <c r="H1" s="6" t="inlineStr">
         <is>
           <t>Quantita</t>
         </is>
       </c>
-      <c r="I1" s="5" t="inlineStr">
+      <c r="I1" s="6" t="inlineStr">
         <is>
           <t>Acquisto</t>
         </is>
       </c>
-      <c r="J1" s="5" t="inlineStr">
+      <c r="J1" s="6" t="inlineStr">
         <is>
           <t>Vendita</t>
         </is>
       </c>
-      <c r="K1" s="5" t="inlineStr">
+      <c r="K1" s="6" t="inlineStr">
         <is>
           <t>Val. iniz. orig.</t>
         </is>
       </c>
-      <c r="L1" s="5" t="inlineStr">
+      <c r="L1" s="6" t="inlineStr">
         <is>
           <t>Val. fin. orig.</t>
         </is>
       </c>
-      <c r="M1" s="5" t="inlineStr">
+      <c r="M1" s="6" t="inlineStr">
         <is>
           <t>Cambio iniz.</t>
         </is>
       </c>
-      <c r="N1" s="5" t="inlineStr">
+      <c r="N1" s="6" t="inlineStr">
         <is>
           <t>Cambio fin.</t>
         </is>
       </c>
-      <c r="O1" s="5" t="inlineStr">
+      <c r="O1" s="6" t="inlineStr">
         <is>
           <t>Val. iniz. EUR</t>
         </is>
       </c>
-      <c r="P1" s="5" t="inlineStr">
+      <c r="P1" s="6" t="inlineStr">
         <is>
           <t>Val. fin. EUR</t>
         </is>
       </c>
-      <c r="Q1" s="5" t="inlineStr">
+      <c r="Q1" s="6" t="inlineStr">
         <is>
           <t>Giorni</t>
         </is>
       </c>
-      <c r="R1" s="5" t="inlineStr">
+      <c r="R1" s="6" t="inlineStr">
         <is>
           <t>Quota %</t>
         </is>
       </c>
-      <c r="S1" s="5" t="inlineStr">
+      <c r="S1" s="6" t="inlineStr">
         <is>
           <t>IVAFE</t>
         </is>
@@ -1680,7 +1725,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="S15" s="6" t="n"/>
+      <c r="S15" s="7" t="n"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr"/>
@@ -1739,67 +1784,67 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>Simbolo</t>
         </is>
       </c>
-      <c r="B1" s="5" t="inlineStr">
+      <c r="B1" s="6" t="inlineStr">
         <is>
           <t>ISIN</t>
         </is>
       </c>
-      <c r="C1" s="5" t="inlineStr">
+      <c r="C1" s="6" t="inlineStr">
         <is>
           <t>Azienda</t>
         </is>
       </c>
-      <c r="D1" s="5" t="inlineStr">
+      <c r="D1" s="6" t="inlineStr">
         <is>
           <t>Data acquisto</t>
         </is>
       </c>
-      <c r="E1" s="5" t="inlineStr">
+      <c r="E1" s="6" t="inlineStr">
         <is>
           <t>Data vendita</t>
         </is>
       </c>
-      <c r="F1" s="5" t="inlineStr">
+      <c r="F1" s="6" t="inlineStr">
         <is>
           <t>Quantita</t>
         </is>
       </c>
-      <c r="G1" s="5" t="inlineStr">
+      <c r="G1" s="6" t="inlineStr">
         <is>
           <t>Corrispettivo EUR</t>
         </is>
       </c>
-      <c r="H1" s="5" t="inlineStr">
+      <c r="H1" s="6" t="inlineStr">
         <is>
           <t>Costo EUR</t>
         </is>
       </c>
-      <c r="I1" s="5" t="inlineStr">
+      <c r="I1" s="6" t="inlineStr">
         <is>
           <t>+/- EUR</t>
         </is>
       </c>
-      <c r="J1" s="5" t="inlineStr">
+      <c r="J1" s="6" t="inlineStr">
         <is>
           <t>Cambio BCE</t>
         </is>
       </c>
-      <c r="K1" s="5" t="inlineStr">
+      <c r="K1" s="6" t="inlineStr">
         <is>
           <t>Forex</t>
         </is>
       </c>
-      <c r="L1" s="5" t="inlineStr">
+      <c r="L1" s="6" t="inlineStr">
         <is>
           <t>P/L broker</t>
         </is>
       </c>
-      <c r="M1" s="5" t="inlineStr">
+      <c r="M1" s="6" t="inlineStr">
         <is>
           <t>P/L broker EUR</t>
         </is>
@@ -2116,7 +2161,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="I8" s="6" t="n"/>
+      <c r="I8" s="7" t="n"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr"/>
@@ -2159,37 +2204,37 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>Descrizione</t>
         </is>
       </c>
-      <c r="B1" s="5" t="inlineStr">
+      <c r="B1" s="6" t="inlineStr">
         <is>
           <t>Valuta</t>
         </is>
       </c>
-      <c r="C1" s="5" t="inlineStr">
+      <c r="C1" s="6" t="inlineStr">
         <is>
           <t>Lordo</t>
         </is>
       </c>
-      <c r="D1" s="5" t="inlineStr">
+      <c r="D1" s="6" t="inlineStr">
         <is>
           <t>Lordo EUR</t>
         </is>
       </c>
-      <c r="E1" s="5" t="inlineStr">
+      <c r="E1" s="6" t="inlineStr">
         <is>
           <t>Ritenuta</t>
         </is>
       </c>
-      <c r="F1" s="5" t="inlineStr">
+      <c r="F1" s="6" t="inlineStr">
         <is>
           <t>Ritenuta EUR</t>
         </is>
       </c>
-      <c r="G1" s="5" t="inlineStr">
+      <c r="G1" s="6" t="inlineStr">
         <is>
           <t>Netto EUR</t>
         </is>
@@ -2331,9 +2376,9 @@
       </c>
     </row>
     <row r="7">
-      <c r="D7" s="6" t="n"/>
-      <c r="F7" s="6" t="n"/>
-      <c r="G7" s="6" t="n"/>
+      <c r="D7" s="7" t="n"/>
+      <c r="F7" s="7" t="n"/>
+      <c r="G7" s="7" t="n"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr"/>
@@ -2410,32 +2455,32 @@
     </row>
     <row r="3"/>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" s="6" t="inlineStr">
         <is>
           <t>Data</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>Saldo USD</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>Equiv. EUR</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="6" t="inlineStr">
         <is>
           <t>Cambio</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E4" s="6" t="inlineStr">
         <is>
           <t>Giorno lavorativo</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="F4" s="6" t="inlineStr">
         <is>
           <t>Sopra soglia</t>
         </is>

</xml_diff>